<commit_message>
chore: added test documents and test sets
</commit_message>
<xml_diff>
--- a/test/data-driven/nearest_stars.xlsx
+++ b/test/data-driven/nearest_stars.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alessandrabelen/Documents/table_aware/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alessandrabelen/Documents/rag_system_v2/rag_system/test/data-driven/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC547F80-543D-3D4F-9B3D-31252E24B4F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D1FE36F-C4BD-BC41-94D3-C5EAF167C73F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28800" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{94C12D85-FB9D-0D46-A41B-A1F71A9F6996}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="343">
   <si>
     <t>HIP</t>
   </si>
@@ -407,12 +407,783 @@
   <si>
     <t>B-V (mag)</t>
   </si>
+  <si>
+    <t>Wolf 1061</t>
+  </si>
+  <si>
+    <t>10.1</t>
+  </si>
+  <si>
+    <t>11.95</t>
+  </si>
+  <si>
+    <t>M4</t>
+  </si>
+  <si>
+    <t>8.56</t>
+  </si>
+  <si>
+    <t>10.36</t>
+  </si>
+  <si>
+    <t>12.16</t>
+  </si>
+  <si>
+    <t>13.94</t>
+  </si>
+  <si>
+    <t>van Maanen's Star</t>
+  </si>
+  <si>
+    <t>12.37</t>
+  </si>
+  <si>
+    <t>14.15</t>
+  </si>
+  <si>
+    <t>0.554</t>
+  </si>
+  <si>
+    <t>DG</t>
+  </si>
+  <si>
+    <t>12.07</t>
+  </si>
+  <si>
+    <t>13.80</t>
+  </si>
+  <si>
+    <t>9.15</t>
+  </si>
+  <si>
+    <t>10.87</t>
+  </si>
+  <si>
+    <t>M3.5Vvar</t>
+  </si>
+  <si>
+    <t>9.38</t>
+  </si>
+  <si>
+    <t>11.10</t>
+  </si>
+  <si>
+    <t>12.24</t>
+  </si>
+  <si>
+    <t>13.92</t>
+  </si>
+  <si>
+    <t>11.5</t>
+  </si>
+  <si>
+    <t>13.18</t>
+  </si>
+  <si>
+    <t>0.196</t>
+  </si>
+  <si>
+    <t>DC:</t>
+  </si>
+  <si>
+    <t>IL Aquarii or Ross 780</t>
+  </si>
+  <si>
+    <t>10.16</t>
+  </si>
+  <si>
+    <t>11.80</t>
+  </si>
+  <si>
+    <t>Furuhjelm I- 650</t>
+  </si>
+  <si>
+    <t>8.82</t>
+  </si>
+  <si>
+    <t>10.40</t>
+  </si>
+  <si>
+    <t>M2Vvar</t>
+  </si>
+  <si>
+    <t>6.6</t>
+  </si>
+  <si>
+    <t>8.16</t>
+  </si>
+  <si>
+    <t>K8V</t>
+  </si>
+  <si>
+    <t>13.26</t>
+  </si>
+  <si>
+    <t>11.39</t>
+  </si>
+  <si>
+    <t>12.92</t>
+  </si>
+  <si>
+    <t>8.66</t>
+  </si>
+  <si>
+    <t>10.19</t>
+  </si>
+  <si>
+    <t>10.94</t>
+  </si>
+  <si>
+    <t>12.43</t>
+  </si>
+  <si>
+    <r>
+      <t>o</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times"/>
+      </rPr>
+      <t xml:space="preserve"> Eridani A</t>
+    </r>
+  </si>
+  <si>
+    <t>4.43</t>
+  </si>
+  <si>
+    <t>5.92</t>
+  </si>
+  <si>
+    <t>0.82</t>
+  </si>
+  <si>
+    <t>EV Lacertae</t>
+  </si>
+  <si>
+    <t>10.29</t>
+  </si>
+  <si>
+    <t>11.77</t>
+  </si>
+  <si>
+    <t>1.54</t>
+  </si>
+  <si>
+    <t>70 Ophiuchi A</t>
+  </si>
+  <si>
+    <t>4.03</t>
+  </si>
+  <si>
+    <t>5.50</t>
+  </si>
+  <si>
+    <t>0.86</t>
+  </si>
+  <si>
+    <t>K0V SB</t>
+  </si>
+  <si>
+    <t>Altair</t>
+  </si>
+  <si>
+    <t>0.76</t>
+  </si>
+  <si>
+    <t>2.20</t>
+  </si>
+  <si>
+    <t>0.221</t>
+  </si>
+  <si>
+    <t>A7IV-V</t>
+  </si>
+  <si>
+    <t>11.49</t>
+  </si>
+  <si>
+    <t>12.90</t>
+  </si>
+  <si>
+    <t>1.75</t>
+  </si>
+  <si>
+    <t>M:</t>
+  </si>
+  <si>
+    <t>10.8</t>
+  </si>
+  <si>
+    <t>12.14</t>
+  </si>
+  <si>
+    <t>Wolf 498</t>
+  </si>
+  <si>
+    <t>8.46</t>
+  </si>
+  <si>
+    <t>9.79</t>
+  </si>
+  <si>
+    <t>M3V</t>
+  </si>
+  <si>
+    <t>11.41</t>
+  </si>
+  <si>
+    <t>12.71</t>
+  </si>
+  <si>
+    <t>10.82</t>
+  </si>
+  <si>
+    <t>12.11</t>
+  </si>
+  <si>
+    <t>1.17</t>
+  </si>
+  <si>
+    <t>Wolf 294</t>
+  </si>
+  <si>
+    <t>9.89</t>
+  </si>
+  <si>
+    <t>1.58</t>
+  </si>
+  <si>
+    <t>K:...</t>
+  </si>
+  <si>
+    <t>EE Leo or Wolf 358</t>
+  </si>
+  <si>
+    <t>11.64</t>
+  </si>
+  <si>
+    <t>12.89</t>
+  </si>
+  <si>
+    <t>M4:</t>
+  </si>
+  <si>
+    <t>Wolf 1453</t>
+  </si>
+  <si>
+    <t>7.97</t>
+  </si>
+  <si>
+    <t>9.19</t>
+  </si>
+  <si>
+    <t>Wolf 630</t>
+  </si>
+  <si>
+    <t>9.02</t>
+  </si>
+  <si>
+    <t>10.23</t>
+  </si>
+  <si>
+    <t>M3Ve</t>
+  </si>
+  <si>
+    <r>
+      <t>s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times"/>
+      </rPr>
+      <t xml:space="preserve"> Draconis</t>
+    </r>
+  </si>
+  <si>
+    <t>4.67</t>
+  </si>
+  <si>
+    <t>5.87</t>
+  </si>
+  <si>
+    <t>0.786</t>
+  </si>
+  <si>
+    <t>K0V</t>
+  </si>
+  <si>
+    <t>8.15</t>
+  </si>
+  <si>
+    <t>9.34</t>
+  </si>
+  <si>
+    <t>Ross 47</t>
+  </si>
+  <si>
+    <t>11.56</t>
+  </si>
+  <si>
+    <t>12.75</t>
+  </si>
+  <si>
+    <t>10.75</t>
+  </si>
+  <si>
+    <t>11.93</t>
+  </si>
+  <si>
+    <t>1.66</t>
+  </si>
+  <si>
+    <t>Wolf 1055</t>
+  </si>
+  <si>
+    <t>9.12</t>
+  </si>
+  <si>
+    <t>10.28</t>
+  </si>
+  <si>
+    <t>M3.5V</t>
+  </si>
+  <si>
+    <t>5.72</t>
+  </si>
+  <si>
+    <t>6.86</t>
+  </si>
+  <si>
+    <t>K4V</t>
+  </si>
+  <si>
+    <t>Ross 882</t>
+  </si>
+  <si>
+    <t>11.19</t>
+  </si>
+  <si>
+    <t>12.32</t>
+  </si>
+  <si>
+    <t>1.6</t>
+  </si>
+  <si>
+    <t>9.31</t>
+  </si>
+  <si>
+    <t>10.44</t>
+  </si>
+  <si>
+    <t>M0</t>
+  </si>
+  <si>
+    <r>
+      <t>h</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times"/>
+      </rPr>
+      <t xml:space="preserve"> Cassiopei or Wolf 24</t>
+    </r>
+  </si>
+  <si>
+    <t>3.46</t>
+  </si>
+  <si>
+    <t>4.59</t>
+  </si>
+  <si>
+    <t>0.587</t>
+  </si>
+  <si>
+    <t>G0V SB</t>
+  </si>
+  <si>
+    <t>36 Ophiuchi C</t>
+  </si>
+  <si>
+    <t>6.33</t>
+  </si>
+  <si>
+    <t>7.45</t>
+  </si>
+  <si>
+    <t>BR Piscium</t>
+  </si>
+  <si>
+    <t>8.98</t>
+  </si>
+  <si>
+    <t>10.10</t>
+  </si>
+  <si>
+    <t>1.46</t>
+  </si>
+  <si>
+    <t>36 Ophiuchi</t>
+  </si>
+  <si>
+    <t>4.33</t>
+  </si>
+  <si>
+    <t>5.44</t>
+  </si>
+  <si>
+    <t>0.855</t>
+  </si>
+  <si>
+    <t>K2:III:</t>
+  </si>
+  <si>
+    <t>5.32</t>
+  </si>
+  <si>
+    <t>6.41</t>
+  </si>
+  <si>
+    <t>0.868</t>
+  </si>
+  <si>
+    <t>82 Eridani</t>
+  </si>
+  <si>
+    <t>4.26</t>
+  </si>
+  <si>
+    <t>5.35</t>
+  </si>
+  <si>
+    <t>0.711</t>
+  </si>
+  <si>
+    <r>
+      <t>d</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times"/>
+      </rPr>
+      <t xml:space="preserve"> Pavonis</t>
+    </r>
+  </si>
+  <si>
+    <t>3.55</t>
+  </si>
+  <si>
+    <t>4.62</t>
+  </si>
+  <si>
+    <t>0.751</t>
+  </si>
+  <si>
+    <t>G5IV-Vvar</t>
+  </si>
+  <si>
+    <t>Wolf 1481</t>
+  </si>
+  <si>
+    <t>11.32</t>
+  </si>
+  <si>
+    <t>12.39</t>
+  </si>
+  <si>
+    <t>10.49</t>
+  </si>
+  <si>
+    <t>11.53</t>
+  </si>
+  <si>
+    <t>M2V:</t>
+  </si>
+  <si>
+    <t>7.64</t>
+  </si>
+  <si>
+    <t>8.68</t>
+  </si>
+  <si>
+    <t>1.41</t>
+  </si>
+  <si>
+    <t>9.01</t>
+  </si>
+  <si>
+    <t>EQ Pegasi</t>
+  </si>
+  <si>
+    <t>10.05</t>
+  </si>
+  <si>
+    <t>11.07</t>
+  </si>
+  <si>
+    <t>1.19</t>
+  </si>
+  <si>
+    <t>M6Ve</t>
+  </si>
+  <si>
+    <t>HO Librae or Wolf 562</t>
+  </si>
+  <si>
+    <t>10.57</t>
+  </si>
+  <si>
+    <t>7.7</t>
+  </si>
+  <si>
+    <t>1.42</t>
+  </si>
+  <si>
+    <t>K2</t>
+  </si>
+  <si>
+    <t>10.31</t>
+  </si>
+  <si>
+    <t>QY Aurigae or Ross 986</t>
+  </si>
+  <si>
+    <t>11.65</t>
+  </si>
+  <si>
+    <t>12.63</t>
+  </si>
+  <si>
+    <t>1.7</t>
+  </si>
+  <si>
+    <t>11.69</t>
+  </si>
+  <si>
+    <t>12.65</t>
+  </si>
+  <si>
+    <t>Wolf 629</t>
+  </si>
+  <si>
+    <t>11.73</t>
+  </si>
+  <si>
+    <t>12.67</t>
+  </si>
+  <si>
+    <t>5.57</t>
+  </si>
+  <si>
+    <t>6.50</t>
+  </si>
+  <si>
+    <t>K3Vvar</t>
+  </si>
+  <si>
+    <t>10.13</t>
+  </si>
+  <si>
+    <t>11.04</t>
+  </si>
+  <si>
+    <t>M2</t>
+  </si>
+  <si>
+    <t>Ross 104</t>
+  </si>
+  <si>
+    <t>10.03</t>
+  </si>
+  <si>
+    <t>10.92</t>
+  </si>
+  <si>
+    <t>M3</t>
+  </si>
+  <si>
+    <t>37 Bootis</t>
+  </si>
+  <si>
+    <t>4.54</t>
+  </si>
+  <si>
+    <t>5.41</t>
+  </si>
+  <si>
+    <t>0.72</t>
+  </si>
+  <si>
+    <t>G8V + K4V</t>
+  </si>
+  <si>
+    <t>Ross 775</t>
+  </si>
+  <si>
+    <t>1.62</t>
+  </si>
+  <si>
+    <t>12.28</t>
+  </si>
+  <si>
+    <t>13.13</t>
+  </si>
+  <si>
+    <t>Ross 671</t>
+  </si>
+  <si>
+    <t>9.49</t>
+  </si>
+  <si>
+    <t>M2:</t>
+  </si>
+  <si>
+    <t>5.91</t>
+  </si>
+  <si>
+    <t>8.55</t>
+  </si>
+  <si>
+    <t>5.79</t>
+  </si>
+  <si>
+    <t>0.918</t>
+  </si>
+  <si>
+    <t>K3V</t>
+  </si>
+  <si>
+    <t>Ross 446</t>
+  </si>
+  <si>
+    <t>9.65</t>
+  </si>
+  <si>
+    <t>10.35</t>
+  </si>
+  <si>
+    <t>12.47</t>
+  </si>
+  <si>
+    <t>Wolf 25</t>
+  </si>
+  <si>
+    <t>5.74</t>
+  </si>
+  <si>
+    <t>6.38</t>
+  </si>
+  <si>
+    <t>0.89</t>
+  </si>
+  <si>
+    <t>107 Piscium</t>
+  </si>
+  <si>
+    <t>5.24</t>
+  </si>
+  <si>
+    <t>0.836</t>
+  </si>
+  <si>
+    <r>
+      <t>b</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times"/>
+      </rPr>
+      <t xml:space="preserve"> Hydri</t>
+    </r>
+  </si>
+  <si>
+    <t>2.82</t>
+  </si>
+  <si>
+    <t>3.45</t>
+  </si>
+  <si>
+    <t>0.618</t>
+  </si>
+  <si>
+    <t>G2IV</t>
+  </si>
+  <si>
+    <t>8.01</t>
+  </si>
+  <si>
+    <t>8.64</t>
+  </si>
+  <si>
+    <t>VX Arietis or Ross 556</t>
+  </si>
+  <si>
+    <t>10.55</t>
+  </si>
+  <si>
+    <t>11.16</t>
+  </si>
+  <si>
+    <t>1.53</t>
+  </si>
+  <si>
+    <r>
+      <t>m</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times"/>
+      </rPr>
+      <t xml:space="preserve"> Cassiopei A</t>
+    </r>
+  </si>
+  <si>
+    <t>5.17</t>
+  </si>
+  <si>
+    <t>5.78</t>
+  </si>
+  <si>
+    <t>0.704</t>
+  </si>
+  <si>
+    <t>G5Vp</t>
+  </si>
+  <si>
+    <t>Ross 490</t>
+  </si>
+  <si>
+    <t>9.05</t>
+  </si>
+  <si>
+    <t>9.64</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -437,6 +1208,12 @@
       <name val="Symbol"/>
       <charset val="2"/>
     </font>
+    <font>
+      <vertAlign val="superscript"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -458,13 +1235,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -799,14 +1575,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB75EACB-C80F-DF4F-988F-EE2B64DD3D7D}">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.33203125" style="3" customWidth="1"/>
-    <col min="3" max="4" width="10.83203125" style="3"/>
-    <col min="5" max="6" width="11" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="10.83203125" style="3"/>
+    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.33203125" customWidth="1"/>
+    <col min="5" max="6" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -822,579 +1596,2206 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="4">
+      <c r="A2" s="2">
         <v>70890</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="2">
         <v>12948</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="2">
         <v>1807</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="4">
+      <c r="A3" s="2">
         <v>71681</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="2">
         <v>13475</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="4">
+      <c r="A4" s="2">
         <v>71683</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="2">
         <v>13475</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="4">
+      <c r="A5" s="2">
         <v>87937</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="2">
         <v>18215</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="4">
+      <c r="A6" s="2">
         <v>54035</v>
       </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4" t="s">
+      <c r="B6" s="2"/>
+      <c r="C6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="2">
         <v>25484</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="2">
         <v>1502</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" s="4">
+      <c r="A7" s="2">
         <v>32349</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="2">
         <v>26371</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:7">
-      <c r="A8" s="4">
+      <c r="A8" s="2">
         <v>92403</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="2">
         <v>29719</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="2" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" s="4">
+      <c r="A9" s="2">
         <v>16537</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="2">
         <v>32180</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="2" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:7">
-      <c r="A10" s="4">
+      <c r="A10" s="2">
         <v>114046</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="2">
         <v>32906</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="2">
         <v>1483</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="4">
+      <c r="A11" s="2">
         <v>57548</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="2">
         <v>33380</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="2">
         <v>1746</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="2" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="4">
+      <c r="A12" s="2">
         <v>104214</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="2">
         <v>34827</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="2">
         <v>1069</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="2" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="4">
+      <c r="A13" s="2">
         <v>37279</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E13" s="2">
         <v>34974</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="2" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="4">
+      <c r="A14" s="2">
         <v>104217</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E14" s="2">
         <v>35036</v>
       </c>
-      <c r="F14" s="4">
+      <c r="F14" s="2">
         <v>1309</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="2" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="4">
+      <c r="A15" s="2">
         <v>91772</v>
       </c>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4" t="s">
+      <c r="B15" s="2"/>
+      <c r="C15" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="2">
         <v>35152</v>
       </c>
-      <c r="F15" s="4">
+      <c r="F15" s="2">
         <v>1561</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="2" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="4">
+      <c r="A16" s="2">
         <v>91768</v>
       </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4" t="s">
+      <c r="B16" s="2"/>
+      <c r="C16" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E16" s="2">
         <v>35679</v>
       </c>
-      <c r="F16" s="4">
+      <c r="F16" s="2">
         <v>1504</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="2" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="4">
+      <c r="A17" s="2">
         <v>1475</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="2">
         <v>35680</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F17" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="G17" s="2" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:7">
-      <c r="A18" s="4">
+      <c r="A18" s="2">
         <v>108870</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E18" s="4">
+      <c r="E18" s="2">
         <v>36263</v>
       </c>
-      <c r="F18" s="4">
+      <c r="F18" s="2">
         <v>1056</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="2" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:7">
-      <c r="A19" s="4">
+      <c r="A19" s="2">
         <v>8102</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="2">
         <v>36474</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="G19" s="2" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="4">
+      <c r="A20" s="2">
         <v>5643</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E20" s="2">
         <v>37168</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="G20" s="2" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="21" spans="1:7">
-      <c r="A21" s="4">
+      <c r="A21" s="2">
         <v>36208</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E21" s="4">
+      <c r="E21" s="2">
         <v>37985</v>
       </c>
-      <c r="F21" s="4">
+      <c r="F21" s="2">
         <v>1573</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="G21" s="2" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="4">
+      <c r="A22" s="2">
         <v>24186</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="E22" s="4">
+      <c r="E22" s="2">
         <v>39176</v>
       </c>
-      <c r="F22" s="4">
+      <c r="F22" s="2">
         <v>1543</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="2" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="4">
+      <c r="A23" s="2">
         <v>105090</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E23" s="4">
+      <c r="E23" s="2">
         <v>39468</v>
       </c>
-      <c r="F23" s="4">
+      <c r="F23" s="2">
         <v>1397</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="G23" s="2" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="4">
+      <c r="A24" s="2">
         <v>110893</v>
       </c>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4" t="s">
+      <c r="B24" s="2"/>
+      <c r="C24" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E24" s="4">
+      <c r="E24" s="2">
         <v>40077</v>
       </c>
-      <c r="F24" s="4">
+      <c r="F24" s="2">
         <v>1613</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="G24" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="25" spans="1:7">
-      <c r="A25" s="4">
+      <c r="A25" s="2">
         <v>30920</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E25" s="4">
+      <c r="E25" s="2">
         <v>41171</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="F25" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="G25" s="2" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="26" spans="1:7">
-      <c r="A26" s="4">
+      <c r="A26" s="2">
         <v>72511</v>
       </c>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4" t="s">
+      <c r="B26" s="2"/>
+      <c r="C26" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="E26" s="4">
+      <c r="E26" s="2">
         <v>42510</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="2" t="s">
         <v>105</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="2">
+        <v>80824</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E27" s="4">
+        <v>42642</v>
+      </c>
+      <c r="F27" s="4">
+        <v>1604</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="2">
+        <v>439</v>
+      </c>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E28" s="4">
+        <v>43605</v>
+      </c>
+      <c r="F28" s="4">
+        <v>1462</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="2">
+        <v>15689</v>
+      </c>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E29" s="4">
+        <v>43966</v>
+      </c>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="2">
+        <v>3829</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E30" s="4">
+        <v>44063</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" s="2">
+        <v>72509</v>
+      </c>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E31" s="4">
+        <v>45086</v>
+      </c>
+      <c r="F31" s="4">
+        <v>1524</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="2">
+        <v>86162</v>
+      </c>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E32" s="4">
+        <v>45280</v>
+      </c>
+      <c r="F32" s="4">
+        <v>1505</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" s="2">
+        <v>85523</v>
+      </c>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E33" s="4">
+        <v>45366</v>
+      </c>
+      <c r="F33" s="4">
+        <v>1553</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" s="2">
+        <v>114110</v>
+      </c>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E34" s="4">
+        <v>46185</v>
+      </c>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" s="2">
+        <v>57367</v>
+      </c>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E35" s="4">
+        <v>46211</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" s="2">
+        <v>113020</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E36" s="4">
+        <v>47017</v>
+      </c>
+      <c r="F36" s="4">
+        <v>1597</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" s="2">
+        <v>54211</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E37" s="4">
+        <v>48323</v>
+      </c>
+      <c r="F37" s="4">
+        <v>1491</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" s="2">
+        <v>49908</v>
+      </c>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E38" s="4">
+        <v>48728</v>
+      </c>
+      <c r="F38" s="4">
+        <v>1326</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" s="2">
+        <v>82725</v>
+      </c>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E39" s="4">
+        <v>49259</v>
+      </c>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" s="2">
+        <v>85605</v>
+      </c>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E40" s="4">
+        <v>49336</v>
+      </c>
+      <c r="F40" s="4">
+        <v>1101</v>
+      </c>
+      <c r="G40" s="2"/>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" s="2">
+        <v>106440</v>
+      </c>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E41" s="4">
+        <v>49375</v>
+      </c>
+      <c r="F41" s="4">
+        <v>1521</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42" s="2">
+        <v>86214</v>
+      </c>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E42" s="4">
+        <v>50424</v>
+      </c>
+      <c r="F42" s="4">
+        <v>1655</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="18">
+      <c r="A43" s="2">
+        <v>19849</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E43" s="4">
+        <v>50444</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44" s="2">
+        <v>112460</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E44" s="4">
+        <v>50487</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45" s="2">
+        <v>88601</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="E45" s="4">
+        <v>50860</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
+      <c r="A46" s="2">
+        <v>97649</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="E46" s="4">
+        <v>51430</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
+      <c r="A47" s="2">
+        <v>1242</v>
+      </c>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="E47" s="4">
+        <v>52121</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
+      <c r="A48" s="2">
+        <v>57544</v>
+      </c>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="E48" s="4">
+        <v>53914</v>
+      </c>
+      <c r="F48" s="4">
+        <v>1572</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49" s="2">
+        <v>67155</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E49" s="4">
+        <v>54309</v>
+      </c>
+      <c r="F49" s="4">
+        <v>1435</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
+      <c r="A50" s="2">
+        <v>103039</v>
+      </c>
+      <c r="B50" s="2"/>
+      <c r="C50" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="E50" s="4">
+        <v>54900</v>
+      </c>
+      <c r="F50" s="4">
+        <v>1653</v>
+      </c>
+      <c r="G50" s="2"/>
+    </row>
+    <row r="51" spans="1:7">
+      <c r="A51" s="2">
+        <v>21088</v>
+      </c>
+      <c r="B51" s="2"/>
+      <c r="C51" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="E51" s="4">
+        <v>55139</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="G51" s="2"/>
+    </row>
+    <row r="52" spans="1:7">
+      <c r="A52" s="2">
+        <v>33226</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E52" s="4">
+        <v>55151</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
+      <c r="A53" s="2">
+        <v>53020</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="E53" s="4">
+        <v>56351</v>
+      </c>
+      <c r="F53" s="4">
+        <v>1679</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
+      <c r="A54" s="2">
+        <v>25878</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="E54" s="4">
+        <v>56909</v>
+      </c>
+      <c r="F54" s="4">
+        <v>1474</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
+      <c r="A55" s="2">
+        <v>82817</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="E55" s="4">
+        <v>57395</v>
+      </c>
+      <c r="F55" s="4">
+        <v>1553</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
+      <c r="A56" s="2">
+        <v>96100</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="E56" s="4">
+        <v>57667</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
+      <c r="A57" s="2">
+        <v>29295</v>
+      </c>
+      <c r="B57" s="2"/>
+      <c r="C57" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="E57" s="4">
+        <v>57740</v>
+      </c>
+      <c r="F57" s="4">
+        <v>1487</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7">
+      <c r="A58" s="2">
+        <v>26857</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="E58" s="4">
+        <v>57877</v>
+      </c>
+      <c r="F58" s="4">
+        <v>1675</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7">
+      <c r="A59" s="2">
+        <v>86990</v>
+      </c>
+      <c r="B59" s="2"/>
+      <c r="C59" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E59" s="4">
+        <v>58113</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7">
+      <c r="A60" s="2">
+        <v>94761</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E60" s="4">
+        <v>58734</v>
+      </c>
+      <c r="F60" s="4">
+        <v>1464</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7">
+      <c r="A61" s="2">
+        <v>73184</v>
+      </c>
+      <c r="B61" s="2"/>
+      <c r="C61" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="E61" s="4">
+        <v>59060</v>
+      </c>
+      <c r="F61" s="4">
+        <v>1024</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7">
+      <c r="A62" s="2">
+        <v>37766</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="E62" s="4">
+        <v>59315</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7">
+      <c r="A63" s="2">
+        <v>76074</v>
+      </c>
+      <c r="B63" s="2"/>
+      <c r="C63" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="E63" s="4">
+        <v>59340</v>
+      </c>
+      <c r="F63" s="4">
+        <v>1524</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7">
+      <c r="A64" s="2">
+        <v>3821</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="E64" s="4">
+        <v>59527</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7">
+      <c r="A65" s="2">
+        <v>84478</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="E65" s="4">
+        <v>59680</v>
+      </c>
+      <c r="F65" s="4">
+        <v>1144</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7">
+      <c r="A66" s="2">
+        <v>117473</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E66" s="4">
+        <v>59698</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7">
+      <c r="A67" s="2">
+        <v>84405</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="E67" s="4">
+        <v>59852</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7">
+      <c r="A68" s="2">
+        <v>99461</v>
+      </c>
+      <c r="B68" s="2"/>
+      <c r="C68" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="E68" s="4">
+        <v>60518</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7">
+      <c r="A69" s="2">
+        <v>15510</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="E69" s="4">
+        <v>60599</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7">
+      <c r="A70" s="2">
+        <v>99240</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="E70" s="4">
+        <v>61076</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7">
+      <c r="A71" s="2">
+        <v>71253</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E71" s="4">
+        <v>61158</v>
+      </c>
+      <c r="F71" s="4">
+        <v>1633</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7">
+      <c r="A72" s="2">
+        <v>86961</v>
+      </c>
+      <c r="B72" s="2"/>
+      <c r="C72" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="E72" s="4">
+        <v>61816</v>
+      </c>
+      <c r="F72" s="4">
+        <v>1463</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7">
+      <c r="A73" s="2">
+        <v>86963</v>
+      </c>
+      <c r="B73" s="2"/>
+      <c r="C73" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E73" s="4">
+        <v>61816</v>
+      </c>
+      <c r="F73" s="4">
+        <v>1439</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7">
+      <c r="A74" s="2">
+        <v>45343</v>
+      </c>
+      <c r="B74" s="2"/>
+      <c r="C74" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="E74" s="4">
+        <v>61885</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7">
+      <c r="A75" s="2">
+        <v>99701</v>
+      </c>
+      <c r="B75" s="2"/>
+      <c r="C75" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="E75" s="4">
+        <v>62046</v>
+      </c>
+      <c r="F75" s="4">
+        <v>1431</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7">
+      <c r="A76" s="2">
+        <v>116132</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="E76" s="4">
+        <v>62477</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7">
+      <c r="A77" s="2">
+        <v>74995</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E77" s="4">
+        <v>62688</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7">
+      <c r="A78" s="2">
+        <v>120005</v>
+      </c>
+      <c r="B78" s="2"/>
+      <c r="C78" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E78" s="4">
+        <v>62704</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7">
+      <c r="A79" s="2">
+        <v>84140</v>
+      </c>
+      <c r="B79" s="2"/>
+      <c r="C79" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="E79" s="4">
+        <v>63223</v>
+      </c>
+      <c r="F79" s="4">
+        <v>1485</v>
+      </c>
+      <c r="G79" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7">
+      <c r="A80" s="2">
+        <v>34603</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="E80" s="4">
+        <v>63597</v>
+      </c>
+      <c r="F80" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="G80" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7">
+      <c r="A81" s="2">
+        <v>54298</v>
+      </c>
+      <c r="B81" s="2"/>
+      <c r="C81" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="E81" s="4">
+        <v>64400</v>
+      </c>
+      <c r="F81" s="2"/>
+      <c r="G81" s="2"/>
+    </row>
+    <row r="82" spans="1:7">
+      <c r="A82" s="2">
+        <v>82809</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="E82" s="4">
+        <v>64952</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="G82" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7">
+      <c r="A83" s="2">
+        <v>114622</v>
+      </c>
+      <c r="B83" s="2"/>
+      <c r="C83" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="E83" s="4">
+        <v>65257</v>
+      </c>
+      <c r="F83" s="2">
+        <v>1</v>
+      </c>
+      <c r="G83" s="2" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7">
+      <c r="A84" s="2">
+        <v>80459</v>
+      </c>
+      <c r="B84" s="2"/>
+      <c r="C84" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="E84" s="4">
+        <v>65820</v>
+      </c>
+      <c r="F84" s="4">
+        <v>1591</v>
+      </c>
+      <c r="G84" s="2" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7">
+      <c r="A85" s="2">
+        <v>53767</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="E85" s="4">
+        <v>66243</v>
+      </c>
+      <c r="F85" s="4">
+        <v>1525</v>
+      </c>
+      <c r="G85" s="2" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7">
+      <c r="A86" s="2">
+        <v>72659</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="E86" s="4">
+        <v>66997</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="G86" s="2" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7">
+      <c r="A87" s="2">
+        <v>106106</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="E87" s="4">
+        <v>67435</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="G87" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7">
+      <c r="A88" s="2">
+        <v>114176</v>
+      </c>
+      <c r="B88" s="2"/>
+      <c r="C88" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="E88" s="4">
+        <v>67590</v>
+      </c>
+      <c r="F88" s="2"/>
+      <c r="G88" s="2"/>
+    </row>
+    <row r="89" spans="1:7">
+      <c r="A89" s="2">
+        <v>113296</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="E89" s="4">
+        <v>68837</v>
+      </c>
+      <c r="F89" s="4">
+        <v>1507</v>
+      </c>
+      <c r="G89" s="2" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7">
+      <c r="A90" s="2">
+        <v>84709</v>
+      </c>
+      <c r="B90" s="2"/>
+      <c r="C90" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E90" s="4">
+        <v>69711</v>
+      </c>
+      <c r="F90" s="4">
+        <v>1082</v>
+      </c>
+      <c r="G90" s="2" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7">
+      <c r="A91" s="2">
+        <v>103096</v>
+      </c>
+      <c r="B91" s="2"/>
+      <c r="C91" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="E91" s="4">
+        <v>70447</v>
+      </c>
+      <c r="F91" s="4">
+        <v>1483</v>
+      </c>
+      <c r="G91" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7">
+      <c r="A92" s="2">
+        <v>12114</v>
+      </c>
+      <c r="B92" s="2"/>
+      <c r="C92" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="E92" s="4">
+        <v>72088</v>
+      </c>
+      <c r="F92" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="G92" s="2" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7">
+      <c r="A93" s="2">
+        <v>51317</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="E93" s="4">
+        <v>72312</v>
+      </c>
+      <c r="F93" s="4">
+        <v>1507</v>
+      </c>
+      <c r="G93" s="2" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7">
+      <c r="A94" s="2">
+        <v>83945</v>
+      </c>
+      <c r="B94" s="2"/>
+      <c r="C94" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="E94" s="4">
+        <v>72548</v>
+      </c>
+      <c r="F94" s="4">
+        <v>1696</v>
+      </c>
+      <c r="G94" s="2" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7">
+      <c r="A95" s="2">
+        <v>3765</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="E95" s="4">
+        <v>74605</v>
+      </c>
+      <c r="F95" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="G95" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7">
+      <c r="A96" s="2">
+        <v>7981</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="E96" s="4">
+        <v>74677</v>
+      </c>
+      <c r="F96" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="G96" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7">
+      <c r="A97" s="2">
+        <v>2021</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="D97" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="E97" s="4">
+        <v>74750</v>
+      </c>
+      <c r="F97" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="G97" s="2" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7">
+      <c r="A98" s="2">
+        <v>73182</v>
+      </c>
+      <c r="B98" s="2"/>
+      <c r="C98" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="E98" s="4">
+        <v>74833</v>
+      </c>
+      <c r="F98" s="4">
+        <v>1519</v>
+      </c>
+      <c r="G98" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7">
+      <c r="A99" s="2">
+        <v>12781</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="E99" s="4">
+        <v>75517</v>
+      </c>
+      <c r="F99" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="G99" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7">
+      <c r="A100" s="2">
+        <v>5336</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E100" s="4">
+        <v>75529</v>
+      </c>
+      <c r="F100" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="G100" s="2" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7">
+      <c r="A101" s="2">
+        <v>65859</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="E101" s="4">
+        <v>76266</v>
+      </c>
+      <c r="F101" s="4">
+        <v>1493</v>
+      </c>
+      <c r="G101" s="2" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>